<commit_message>
health impact + other changes
</commit_message>
<xml_diff>
--- a/results/results_diabetes_korea_simple_CAPPED.xlsx
+++ b/results/results_diabetes_korea_simple_CAPPED.xlsx
@@ -640,76 +640,76 @@
         <v>11465.14910195645</v>
       </c>
       <c r="U2">
-        <v>0.5468342732675411</v>
+        <v>0.5626339226910462</v>
       </c>
       <c r="V2">
-        <v>0.1230068841019617</v>
+        <v>0.1280886104065338</v>
       </c>
       <c r="W2">
-        <v>0.7571894554780508</v>
+        <v>0.772171860210397</v>
       </c>
       <c r="X2">
-        <v>2765.887754187223</v>
+        <v>2845.802380971312</v>
       </c>
       <c r="Y2">
-        <v>622.1688197877224</v>
+        <v>647.8721914362479</v>
       </c>
       <c r="Z2">
-        <v>3829.864265807981</v>
+        <v>3905.645268944188</v>
       </c>
       <c r="AA2">
-        <v>327.9857287631385</v>
+        <v>337.4622004908626</v>
       </c>
       <c r="AB2">
-        <v>73.77829901551563</v>
+        <v>76.82626763573489</v>
       </c>
       <c r="AC2">
-        <v>454.15466350118</v>
+        <v>463.140960035594</v>
       </c>
       <c r="AD2">
-        <v>3534.187397499984</v>
+        <v>3638.316941053125</v>
       </c>
       <c r="AE2">
-        <v>761.8226371799839</v>
+        <v>792.6225607539411</v>
       </c>
       <c r="AF2">
-        <v>5939.730529890795</v>
+        <v>6071.02065202613</v>
       </c>
       <c r="AG2">
-        <v>4463.571812799732</v>
+        <v>4591.302964718424</v>
       </c>
       <c r="AH2">
-        <v>1003.932538464221</v>
+        <v>1045.256178325193</v>
       </c>
       <c r="AI2">
-        <v>6867.83710839018</v>
+        <v>7023.549035497175</v>
       </c>
       <c r="AJ2">
-        <v>4318.213547425456</v>
+        <v>4442.979429010519</v>
       </c>
       <c r="AK2">
-        <v>971.3546120321663</v>
+        <v>1011.483734227796</v>
       </c>
       <c r="AL2">
-        <v>5979.335832546297</v>
+        <v>6097.648137116453</v>
       </c>
       <c r="AM2">
-        <v>7886.036904286856</v>
+        <v>8114.317764140971</v>
       </c>
       <c r="AN2">
-        <v>1708.77613265136</v>
+        <v>1779.37003733522</v>
       </c>
       <c r="AO2">
-        <v>11727.27152943065</v>
+        <v>11954.11121717787</v>
       </c>
       <c r="AP2">
-        <v>8802.430707795733</v>
+        <v>9060.469984392526</v>
       </c>
       <c r="AQ2">
-        <v>1944.400772079556</v>
+        <v>2025.056148708639</v>
       </c>
       <c r="AR2">
-        <v>12601.50711886464</v>
+        <v>12859.15632227164</v>
       </c>
     </row>
     <row r="3">
@@ -776,76 +776,76 @@
         <v>17957.83716914366</v>
       </c>
       <c r="U3">
-        <v>0.5570496113494856</v>
+        <v>0.763203335786143</v>
       </c>
       <c r="V3">
-        <v>0.187649500168478</v>
+        <v>0.3072384518700522</v>
       </c>
       <c r="W3">
-        <v>0.7777807203980891</v>
+        <v>0.9301545503078142</v>
       </c>
       <c r="X3">
-        <v>4503.189058149241</v>
+        <v>6169.73576649518</v>
       </c>
       <c r="Y3">
-        <v>1516.958559361976</v>
+        <v>2483.715644917502</v>
       </c>
       <c r="Z3">
-        <v>6287.579343698152</v>
+        <v>7519.369384688371</v>
       </c>
       <c r="AA3">
-        <v>436.2032686633281</v>
+        <v>597.634004120697</v>
       </c>
       <c r="AB3">
-        <v>146.9408176019284</v>
+        <v>240.586142121363</v>
       </c>
       <c r="AC3">
-        <v>609.0489709149276</v>
+        <v>728.3668221640369</v>
       </c>
       <c r="AD3">
-        <v>5354.774938319879</v>
+        <v>7347.742171011835</v>
       </c>
       <c r="AE3">
-        <v>1767.869300135417</v>
+        <v>2846.69701371751</v>
       </c>
       <c r="AF3">
-        <v>8857.201371976022</v>
+        <v>11166.23275331706</v>
       </c>
       <c r="AG3">
-        <v>7200.212603762933</v>
+        <v>9815.938980283803</v>
       </c>
       <c r="AH3">
-        <v>2289.962316690566</v>
+        <v>3749.300015655776</v>
       </c>
       <c r="AI3">
-        <v>11366.62840959124</v>
+        <v>13876.02562812383</v>
       </c>
       <c r="AJ3">
-        <v>7201.559657510604</v>
+        <v>9866.723253176686</v>
       </c>
       <c r="AK3">
-        <v>2425.94024415809</v>
+        <v>3971.990995314109</v>
       </c>
       <c r="AL3">
-        <v>10055.18026453531</v>
+        <v>12025.07523256143</v>
       </c>
       <c r="AM3">
-        <v>12667.3265505709</v>
+        <v>17293.41545589716</v>
       </c>
       <c r="AN3">
-        <v>4266.350013160704</v>
+        <v>6980.689862345132</v>
       </c>
       <c r="AO3">
-        <v>18169.03426244861</v>
+        <v>22476.89932761834</v>
       </c>
       <c r="AP3">
-        <v>14488.1320491846</v>
+        <v>19805.23058118445</v>
       </c>
       <c r="AQ3">
-        <v>4822.265981414587</v>
+        <v>7811.367795505657</v>
       </c>
       <c r="AR3">
-        <v>21063.46575576582</v>
+        <v>25651.80266011236</v>
       </c>
     </row>
   </sheetData>

</xml_diff>